<commit_message>
feat: add invalid numbers check
</commit_message>
<xml_diff>
--- a/contatos.xlsx
+++ b/contatos.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="18">
   <si>
     <t>Nome</t>
   </si>
@@ -47,6 +47,9 @@
   </si>
   <si>
     <t>ADASDA</t>
+  </si>
+  <si>
+    <t>(43) 3341-1775</t>
   </si>
   <si>
     <t>(43) 99837-7239</t>
@@ -114,13 +117,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -436,8 +442,8 @@
     <col min="4" max="4" style="3" width="16.862142857142857" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="3" width="16.862142857142857" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="3" width="16.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="3" width="11.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="4" width="11.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -480,17 +486,17 @@
         <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>9</v>
@@ -499,20 +505,20 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>9</v>
@@ -521,20 +527,20 @@
         <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>9</v>
@@ -543,20 +549,20 @@
         <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>9</v>
@@ -565,20 +571,20 @@
         <v>10</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>9</v>
@@ -587,13 +593,13 @@
         <v>10</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>

</xml_diff>

<commit_message>
feat: add new dashboard and automation mongodb
</commit_message>
<xml_diff>
--- a/contatos.xlsx
+++ b/contatos.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="17">
   <si>
     <t>Nome</t>
   </si>
@@ -40,7 +40,7 @@
     <t>Telefone 5</t>
   </si>
   <si>
-    <t>GABRIEL FERNANDES</t>
+    <t>TESTE1 FERNANDES</t>
   </si>
   <si>
     <t>SADJSAJDAKSJDASJ</t>
@@ -55,19 +55,16 @@
     <t>(43) 99837-7239</t>
   </si>
   <si>
-    <t>ALOÍSIO JOSÉ DA SILVA</t>
-  </si>
-  <si>
-    <t>GABRIEL2 FERNANDES</t>
-  </si>
-  <si>
-    <t>ALOÍSIO2 JOSÉ DA SILVA</t>
-  </si>
-  <si>
-    <t>GABRIEL3 FERNANDES</t>
-  </si>
-  <si>
-    <t>ALOÍSIO3 JOSÉ DA SILVA</t>
+    <t>TESTE2 FERNANDES</t>
+  </si>
+  <si>
+    <t>(43) 99637-2886</t>
+  </si>
+  <si>
+    <t>TESTE3 FERNANDES</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -117,13 +114,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -436,14 +436,14 @@
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="21.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="3" width="16.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="16.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="3" width="16.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="11.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="27.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="23.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="17.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="17.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="4" width="16.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="11.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -488,9 +488,7 @@
       <c r="E2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="F2" s="1"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
@@ -505,11 +503,9 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="E3" s="1"/>
       <c r="F3" s="1" t="s">
         <v>12</v>
       </c>
@@ -518,7 +514,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>9</v>
@@ -529,77 +525,73 @@
       <c r="D4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>12</v>
+      <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>12</v>
+      <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>12</v>
+      <c r="A7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>

</xml_diff>